<commit_message>
chore: update glossary exports
</commit_message>
<xml_diff>
--- a/exports/xlsx/terms.xlsx
+++ b/exports/xlsx/terms.xlsx
@@ -542,6 +542,7 @@
       <c r="B2" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Regular grid based on a Geographic Coordinate Reference System (CRS).</t>
         </is>
       </c>
@@ -584,6 +585,7 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Quality or characteristic of a measurement or observation to accurately represent a specific geographic location, time period, or environmental condition.</t>
         </is>
       </c>
@@ -630,6 +632,7 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Earth Observation data generated by spaceborne missions or instruments owned by public or private organizations.</t>
         </is>
       </c>
@@ -676,6 +679,7 @@
       <c r="B5" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: The smallest aggregation of data which is independently managed (i.e. described, inventoried, retrievable).</t>
         </is>
       </c>
@@ -722,6 +726,7 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>- core
+- to be discussed
 description: Interval between successive observations.</t>
         </is>
       </c>
@@ -775,6 +780,7 @@
       <c r="B7" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Action of permanently and irrecoverably removing all copies of data held by an organization.</t>
         </is>
       </c>
@@ -817,6 +823,7 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>- controversial
+- to be discussed
 description: Type of Observation performed at a significant distance from a Phenomenon.</t>
         </is>
       </c>
@@ -868,6 +875,7 @@
       <c r="B9" t="inlineStr">
         <is>
           <t>- high-impact
+  - to be discussed
 description: Data available for use with a specified (small and application dependent) latency, typically 3 hours for meteorological applications.</t>
         </is>
       </c>
@@ -910,6 +918,7 @@
       <c r="B10" t="inlineStr">
         <is>
           <t>- base
+- to be approved
 description: Value and possibly Uncertainty of a Trait of a specific Entity.</t>
         </is>
       </c>
@@ -972,6 +981,7 @@
       <c r="B11" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Coordinate Reference System (CRS) that has a geodetic Reference frame and an ellipsoidal coordinate system.</t>
         </is>
       </c>
@@ -1018,6 +1028,7 @@
       <c r="B12" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: The act of maintaining information in a correct and independently understandable form over the long term.</t>
         </is>
       </c>
@@ -1065,6 +1076,7 @@
       <c r="B13" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Processes and operations used to ensure data technical and intellectual survival through time.</t>
         </is>
       </c>
@@ -1112,6 +1124,7 @@
       <c r="B14" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Method of working with collections, similar to version control systems used in traditional software development but optimized to allow better processing of data and collaboration in data analytics and research contexts.</t>
         </is>
       </c>
@@ -1154,6 +1167,7 @@
       <c r="B15" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Level of categorical detail of information expressed by the number of classes.</t>
         </is>
       </c>
@@ -1196,7 +1210,7 @@
       <c r="B16" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be discussed</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -1238,6 +1252,7 @@
       <c r="B17" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Property enabling other researchers to conduct an independent study with different data and similar but not identical methods, yet arriving at results that confirm the original study's hypothesis.</t>
         </is>
       </c>
@@ -1280,7 +1295,7 @@
       <c r="B18" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1326,6 +1341,7 @@
       <c r="B19" t="inlineStr">
         <is>
           <t>- core
+- to be discussed
 description: Uncertainty associated with the method of classification.</t>
         </is>
       </c>
@@ -1407,7 +1423,7 @@
       <c r="B21" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1455,6 +1471,7 @@
       <c r="B22" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Frequency at which the product is available to users.</t>
         </is>
       </c>
@@ -1501,6 +1518,7 @@
       <c r="B23" t="inlineStr">
         <is>
           <t>- base
+- to be approved
 description: Something that has separate and distinct existence and objective or conceptual reality.</t>
         </is>
       </c>
@@ -1555,6 +1573,7 @@
       <c r="B24" t="inlineStr">
         <is>
           <t>- base
+- to be approved
 description: Part of any space referenced by an identifier.</t>
         </is>
       </c>
@@ -1597,6 +1616,7 @@
       <c r="B25" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Non-negative interval Quantity of time equal to the difference between the final and initial instants of a time interval.</t>
         </is>
       </c>
@@ -1646,6 +1666,7 @@
       <c r="B26" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Time of the day at which the variable or parameter is observed or simulated by a model.</t>
         </is>
       </c>
@@ -1699,6 +1720,7 @@
       <c r="B27" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Levels of a vertical discretization, e.g. pressure levels in an atmospheric model reanalysis or height levels in a forest biomass EO product.</t>
         </is>
       </c>
@@ -1747,6 +1769,7 @@
       <c r="B28" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Electronic data package distributable to users; content is derived from instrument data via processing involving ancillary and auxiliary data.</t>
         </is>
       </c>
@@ -1797,6 +1820,7 @@
       <c r="B29" t="inlineStr">
         <is>
           <t>- base
+  - to be approved
 description: The result of organisation, interpretation, categorisation, classification, or some other form of processing of Data attaching to it a certain meaning that can be understood by the addressee.</t>
         </is>
       </c>
@@ -1843,6 +1867,7 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: The solid, inanimate outer layer of the Geosphere. For the purposes of Earth Observation, includes soils ('pedosphere').</t>
         </is>
       </c>
@@ -1885,7 +1910,7 @@
       <c r="B31" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1974,6 +1999,7 @@
       <c r="B33" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Indicator providing sufficient information to allow all users to readily evaluate the fitness for purpose of the data or derived product.</t>
         </is>
       </c>
@@ -2016,6 +2042,7 @@
       <c r="B34" t="inlineStr">
         <is>
           <t>- base
+- to be approved
 description: Series of activities that interact to produce a result.</t>
         </is>
       </c>
@@ -2062,6 +2089,7 @@
       <c r="B35" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Standard deviation of the probability distribution describing the spread of possible values in quantitative/continuous data.</t>
         </is>
       </c>
@@ -2104,6 +2132,7 @@
       <c r="B36" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: The width of the smallest linear Feature that is still represented on a map.</t>
         </is>
       </c>
@@ -2146,6 +2175,7 @@
       <c r="B37" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Products and collections that have been superseded by a newer version and are still available, but whose use is discouraged since they will be decommissioned in the future.</t>
         </is>
       </c>
@@ -2188,6 +2218,7 @@
       <c r="B38" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Temporal reference in the form of a label or code that identifies a Period.</t>
         </is>
       </c>
@@ -2234,6 +2265,7 @@
       <c r="B39" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: Minimum time of interval between an Observation being tasked and being performed.</t>
         </is>
       </c>
@@ -2276,7 +2308,8 @@
       <c r="B40" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- source missing
+- to be discussed</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2314,7 +2347,7 @@
       <c r="B41" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -2356,6 +2389,7 @@
       <c r="B42" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Smallest spatial object of interest that may be used for reporting and for which the information should be aggregated.</t>
         </is>
       </c>
@@ -2402,6 +2436,7 @@
       <c r="B43" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Data required for production of an EO Collection (e.g., unenhanced satellite mission data) as well as further processed Level-1 data, or any other pre-processed format meeting program requirements.</t>
         </is>
       </c>
@@ -2444,7 +2479,7 @@
       <c r="B44" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -2490,6 +2525,7 @@
       <c r="B45" t="inlineStr">
         <is>
           <t>- high-impact
+- to be discussed
 description: Process by which governments translate their political vision into programmes and actions to deliver outcomes — desired change in the real world.</t>
         </is>
       </c>
@@ -2532,6 +2568,7 @@
       <c r="B46" t="inlineStr">
         <is>
           <t>- base
+- to be discussed
 - controversial
 description: Place referenced by a single set of coordinates within a coordinate reference system.</t>
         </is>
@@ -2579,6 +2616,7 @@
       <c r="B47" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: The area of the smallest Feature that is still represented on a map.</t>
         </is>
       </c>
@@ -2621,6 +2659,7 @@
       <c r="B48" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Part of the electromagnetic spectrum of specific wavelengths, in remote sensing usually described by central wavelength and bandwidth.</t>
         </is>
       </c>
@@ -2663,6 +2702,7 @@
       <c r="B49" t="inlineStr">
         <is>
           <t>- core
+- to be discussed
 description: Determination of the geographic Position of a point (0D) or linear (1D) Feature.</t>
         </is>
       </c>
@@ -2705,7 +2745,7 @@
       <c r="B50" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C50" t="inlineStr"/>
@@ -2747,6 +2787,7 @@
       <c r="B51" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Provision of objective evidence that a given item fulfils specified requirements.</t>
         </is>
       </c>
@@ -2812,6 +2853,7 @@
       <c r="B52" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Higher-level processing and integration output (indicative level 4 and beyond) that goes beyond basic data processing, often designed for policy or decision-making needs.</t>
         </is>
       </c>
@@ -2856,7 +2898,8 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>- core</t>
+          <t>- core
+- to be defined</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -2890,6 +2933,7 @@
       <c r="B54" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Time period used for reporting and for which the information should be aggregated from the native temporal resolution.</t>
         </is>
       </c>
@@ -2938,6 +2982,7 @@
       <c r="B55" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Concerned with the validity of the results of a particular study, enabling readers to check whether results have been manipulated by reproducing exactly the same study using the same data and methods.</t>
         </is>
       </c>
@@ -2980,7 +3025,7 @@
       <c r="B56" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C56" t="inlineStr"/>
@@ -3022,6 +3067,7 @@
       <c r="B57" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Geopositioning of an Object using a Physical Sensor Model or a True Replacement Model.</t>
         </is>
       </c>
@@ -3072,7 +3118,7 @@
       <c r="B58" t="inlineStr">
         <is>
           <t>- controversial
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
@@ -3114,7 +3160,7 @@
       <c r="B59" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C59" t="inlineStr"/>
@@ -3164,7 +3210,7 @@
       <c r="B60" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be discussed</t>
         </is>
       </c>
       <c r="C60" t="inlineStr"/>
@@ -3206,6 +3252,7 @@
       <c r="B61" t="inlineStr">
         <is>
           <t>- core
+  - to be discussed
 description: Period between the end of sensing of a Phenomenon to the beginning of availability of a specific product.</t>
         </is>
       </c>
@@ -3282,6 +3329,7 @@
       <c r="B63" t="inlineStr">
         <is>
           <t>- core
+- to be discussed
 description: Service to disseminate Data.</t>
         </is>
       </c>
@@ -3324,6 +3372,7 @@
       <c r="B64" t="inlineStr">
         <is>
           <t>- base
+- to be approved
 description: Entity with at least one Property referenced by an identifier.</t>
         </is>
       </c>
@@ -3366,6 +3415,7 @@
       <c r="B65" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Spheres dividing planet Earth into subsystems, which are collectives of (physical) matter sharing specific traits.</t>
         </is>
       </c>
@@ -3419,6 +3469,7 @@
       <c r="B66" t="inlineStr">
         <is>
           <t>- base
+- to be approved
 description: Element of a type domain.</t>
         </is>
       </c>
@@ -3466,6 +3517,7 @@
       <c r="B67" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Period between the moment of requesting information and the moment of availability of information.</t>
         </is>
       </c>
@@ -3516,7 +3568,7 @@
       <c r="B68" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C68" t="inlineStr"/>
@@ -3581,7 +3633,7 @@
       <c r="B69" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C69" t="inlineStr"/>
@@ -3629,6 +3681,7 @@
       <c r="B70" t="inlineStr">
         <is>
           <t>- base
+- to be approved
 description: Property having a magnitude that can be expressed as a number from a continuous and contiguous range and a reference.</t>
         </is>
       </c>
@@ -3679,6 +3732,7 @@
       <c r="B71" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Product within an EO Collection that is not expected to be updated.</t>
         </is>
       </c>
@@ -3725,6 +3779,7 @@
       <c r="B72" t="inlineStr">
         <is>
           <t>- controversial
+  - to be discussed
 description: Act of determining the Value of a Property by interacting in a reproducible way with the Phenomenon using a Sensor.</t>
         </is>
       </c>
@@ -3772,7 +3827,7 @@
       <c r="B73" t="inlineStr">
         <is>
           <t>- base
-- approved</t>
+- to be discussed</t>
         </is>
       </c>
       <c r="C73" t="inlineStr"/>
@@ -3838,6 +3893,7 @@
       <c r="B74" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: The masses of minerals that constitute planet Earth.</t>
         </is>
       </c>
@@ -3880,6 +3936,7 @@
       <c r="B75" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Measure of the ability to resolve features in the electromagnetic spectrum.</t>
         </is>
       </c>
@@ -3922,6 +3979,7 @@
       <c r="B76" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: The masses of liquid water, such as oceans, lakes, and rivers.</t>
         </is>
       </c>
@@ -3964,6 +4022,7 @@
       <c r="B77" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Time of the year at which the variable is observed or simulated by a model.</t>
         </is>
       </c>
@@ -4013,6 +4072,7 @@
       <c r="B78" t="inlineStr">
         <is>
           <t>- base
+- to be approved
 description: "Line defined in an algorithmic way using at least two positions (can be open-ended). Alternative: line connecting two positions in an algorithmic way (limited by end points)."</t>
         </is>
       </c>
@@ -4059,6 +4119,7 @@
       <c r="B79" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Condition where the spatial statistical properties of the data depend only on the underlying physical processes and not on other factors such as fusing different products or sensors.</t>
         </is>
       </c>
@@ -4101,7 +4162,7 @@
       <c r="B80" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C80" t="inlineStr"/>
@@ -4147,7 +4208,7 @@
       <c r="B81" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C81" t="inlineStr"/>
@@ -4189,6 +4250,7 @@
       <c r="B82" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Product additionally processed from baseline or unenhanced mission data.</t>
         </is>
       </c>
@@ -4236,6 +4298,7 @@
       <c r="B83" t="inlineStr">
         <is>
           <t>- high-impact
+- to be discussed
 description: Desired outcome that policymakers wish to achieve.</t>
         </is>
       </c>
@@ -4278,6 +4341,7 @@
       <c r="B84" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Process of assessing, by independent means, the quality of the data products derived from the system outputs.</t>
         </is>
       </c>
@@ -4348,6 +4412,7 @@
       <c r="B85" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Period during which data was collected, observations were made, or for which the model was run.</t>
         </is>
       </c>
@@ -4399,6 +4464,7 @@
       <c r="B86" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Property of a measurement result whereby the result can be related to a reference through a documented unbroken chain of calibrations each contributing to the measurement uncertainty.</t>
         </is>
       </c>
@@ -4441,6 +4507,7 @@
       <c r="B87" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Products and collections that have been superseded by new versions and are no longer available.</t>
         </is>
       </c>
@@ -4487,6 +4554,7 @@
       <c r="B88" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: Network composed of two or more sets of curves in which the members of each set intersect the members of the other sets in an algorithmic way.</t>
         </is>
       </c>
@@ -4534,6 +4602,7 @@
       <c r="B89" t="inlineStr">
         <is>
           <t>- core
+  - to be discussed
 description: Observation of a Quantity.</t>
         </is>
       </c>
@@ -4580,7 +4649,7 @@
       <c r="B90" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C90" t="inlineStr"/>
@@ -4626,6 +4695,7 @@
       <c r="B91" t="inlineStr">
         <is>
           <t>- core
+- to be discussed
 description: Phenomenon whose values for specific properties are known and understood with an Uncertainty significantly lower than that of the Observation with which it is compared.</t>
         </is>
       </c>
@@ -4672,6 +4742,7 @@
       <c r="B92" t="inlineStr">
         <is>
           <t>- core
+  - to be discussed
 description: Usually in-situ observations in which the Object or Phenomenon is isolated from other systems or altered in its original conditions or environment.</t>
         </is>
       </c>
@@ -4718,6 +4789,7 @@
       <c r="B93" t="inlineStr">
         <is>
           <t>- controversial
+- to be discussed
 description: Subset of one or more entities.</t>
         </is>
       </c>
@@ -4766,6 +4838,7 @@
       <c r="B94" t="inlineStr">
         <is>
           <t>- base
+- to be approved
 description: Characteristic belonging to an entity and referenced by an identifier.</t>
         </is>
       </c>
@@ -4812,6 +4885,7 @@
       <c r="B95" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: Data describing other data, providing an understanding of the content and utility of a product or collection.</t>
         </is>
       </c>
@@ -4859,7 +4933,7 @@
       <c r="B96" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C96" t="inlineStr"/>
@@ -4939,7 +5013,7 @@
       <c r="B98" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C98" t="inlineStr"/>
@@ -4985,7 +5059,7 @@
       <c r="B99" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C99" t="inlineStr"/>
@@ -5027,6 +5101,7 @@
       <c r="B100" t="inlineStr">
         <is>
           <t>- core
+  - to be discussed
 description: Regarded long-term according to X. However, in the Horizon Europe Missions terminology, regarded short-term.</t>
         </is>
       </c>
@@ -5069,6 +5144,7 @@
       <c r="B101" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: Products or collections which have been superseded by later versions of a product or collection.</t>
         </is>
       </c>
@@ -5111,6 +5187,7 @@
       <c r="B102" t="inlineStr">
         <is>
           <t>- core
+  - to be discussed
 description: Uncertainty associated with the method of Measurement.</t>
         </is>
       </c>
@@ -5153,6 +5230,7 @@
       <c r="B103" t="inlineStr">
         <is>
           <t>- core
+- to be defined
 description: ''</t>
         </is>
       </c>
@@ -5191,6 +5269,7 @@
       <c r="B104" t="inlineStr">
         <is>
           <t>- controversial
+  - to be discussed
 description: Observations performed in the same Place where a Phenomenon occurs, normally without isolating it from other systems or altering its pre-Observation state.</t>
         </is>
       </c>
@@ -5238,6 +5317,7 @@
       <c r="B105" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Direct output from standardized satellite data processing chains (indicative levels 2 and 3), representing fundamental geophysical and biophysical variables.</t>
         </is>
       </c>
@@ -5285,6 +5365,7 @@
       <c r="B106" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Presence or absence of gaps, which are missing values in an otherwise continuous spatial data series.</t>
         </is>
       </c>
@@ -5331,6 +5412,7 @@
       <c r="B107" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Translation of one form of Location into another.</t>
         </is>
       </c>
@@ -5377,6 +5459,7 @@
       <c r="B108" t="inlineStr">
         <is>
           <t>- core
+  - to be discussed
 description: Correcting for positional displacement with respect to the surface of the Earth.</t>
         </is>
       </c>
@@ -5431,6 +5514,7 @@
       <c r="B109" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Legal instrument by which a copyright holder may grant rights over the protected work.</t>
         </is>
       </c>
@@ -5473,6 +5557,7 @@
       <c r="B110" t="inlineStr">
         <is>
           <t>- base
+- to be approved
 description: Particular era or span of time.</t>
         </is>
       </c>
@@ -5519,7 +5604,7 @@
       <c r="B111" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C111" t="inlineStr"/>
@@ -5561,6 +5646,7 @@
       <c r="B112" t="inlineStr">
         <is>
           <t>- base
+- to be discussed
 description: Abstraction of real-world phenomena.</t>
         </is>
       </c>
@@ -5607,6 +5693,7 @@
       <c r="B113" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Entity responsible for the safe custody, transport, storage of the data and implementation of business rules.</t>
         </is>
       </c>
@@ -5653,7 +5740,7 @@
       <c r="B114" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C114" t="inlineStr"/>
@@ -5695,6 +5782,7 @@
       <c r="B115" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Entity (person, organization, institution, etc.) that is requesting data or information with certain characteristics described by needs and/or requirements.</t>
         </is>
       </c>
@@ -5749,6 +5837,7 @@
       <c r="B116" t="inlineStr">
         <is>
           <t>- core
+- to be discussed
 description: Entity responsible for the safe custody, transport, storage of the data and implementation of business rules.</t>
         </is>
       </c>
@@ -5795,6 +5884,7 @@
       <c r="B117" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Condition where the temporal statistical properties of the sample depend only on the underlying physical processes and not on other factors such as fusing different products or sensors.</t>
         </is>
       </c>
@@ -5837,6 +5927,7 @@
       <c r="B118" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: Data consisting of, derived from, or relating to information that is directly linked to specific geographical locations.</t>
         </is>
       </c>
@@ -5880,6 +5971,7 @@
       <c r="B119" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Maximum acceptable change in Uncertainty per decade.</t>
         </is>
       </c>
@@ -5926,6 +6018,7 @@
       <c r="B120" t="inlineStr">
         <is>
           <t>- base
+- to be discussed
 description: Observable Trait.</t>
         </is>
       </c>
@@ -5968,6 +6061,7 @@
       <c r="B121" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Data with implicit or explicit reference to a Location relative to the Earth.</t>
         </is>
       </c>
@@ -6014,6 +6108,7 @@
       <c r="B122" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Parameter, associated with the result of a measurement, that characterises the dispersion of the values that could reasonably be attributed to the measurand.</t>
         </is>
       </c>
@@ -6097,6 +6192,7 @@
       <c r="B123" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Set of all the components of an interactive system that provide information and controls for the user to accomplish specific tasks with the interactive system.</t>
         </is>
       </c>
@@ -6139,6 +6235,7 @@
       <c r="B124" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: Data specifically associated with the instrument, either because it was generated by the instrument or included in data packets identified with that instrument.</t>
         </is>
       </c>
@@ -6201,6 +6298,7 @@
       <c r="B125" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: Particular Quantity subject to Measurement.</t>
         </is>
       </c>
@@ -6214,7 +6312,8 @@
       <c r="F125" t="inlineStr">
         <is>
           <t>| Step | Process description |
-| :----- | :--------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------- |
+| :----- | :------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------------
+--- |
 | (Raw) | The complete and unaltered/unprocessed set of Data acquired by one or several sensors on a platform |
 | M/0 uncalibrated | Unaltered/unprocessed Level 0 (main) Sensor Data annotated with processed Ancillary Data and supplemented by Auxiliary Data (including radiometric and geometric Calibration coefficients and geo-referencing parameters) allowing further processing to higher Levels. |
 | M/1 Sensor-calibrated | Level M/0 Sensor Data which have been calibrated (ideally traceable to SI) and spatially aligned (co-located, eventually co-gridded) to represent at-Sensor measurements (Value and Uncertainty) in Sensor nominal spatiotemporal sampling, supplemented by appropriate ancillary data. |
@@ -6255,6 +6354,7 @@
       <c r="B126" t="inlineStr">
         <is>
           <t>- high-impact
+- to be discussed
 description: Specific level or rate set for the Policy Objective.</t>
         </is>
       </c>
@@ -6297,6 +6397,7 @@
       <c r="B127" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Zone or region of space described by a geographic identifier in the form of a label or code, or by a bounding box, representing the maximum spatial boundary within which the user is requesting data.</t>
         </is>
       </c>
@@ -6348,6 +6449,7 @@
       <c r="B128" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Products in a research and development phase not yet published into a standardized collection.</t>
         </is>
       </c>
@@ -6390,6 +6492,7 @@
       <c r="B129" t="inlineStr">
         <is>
           <t>- base
+  - to be approved
 description: Entity with a well-defined boundary and identity that encapsulates state and behaviour.</t>
         </is>
       </c>
@@ -6432,6 +6535,7 @@
       <c r="B130" t="inlineStr">
         <is>
           <t>- core
+- to be discussed
 description: The forecast period.</t>
         </is>
       </c>
@@ -6474,6 +6578,7 @@
       <c r="B131" t="inlineStr">
         <is>
           <t>- high-impact
+- to be discussed
 description: Markers of significant progress in addressing specific issues, or crucial decision points where significant choices are made within a policy process.</t>
         </is>
       </c>
@@ -6516,6 +6621,7 @@
       <c r="B132" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Time that an antenna beam spends on a target.</t>
         </is>
       </c>
@@ -6562,6 +6668,7 @@
       <c r="B133" t="inlineStr">
         <is>
           <t>- core
+  - to be approved
 description: Measure of the agreement between the represented Location of an Object and the true Location.</t>
         </is>
       </c>
@@ -6604,6 +6711,7 @@
       <c r="B134" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Standard Uncertainty multiplied by a coverage factor k, chosen to obtain a desired level of confidence.</t>
         </is>
       </c>
@@ -6646,6 +6754,7 @@
       <c r="B135" t="inlineStr">
         <is>
           <t>- core
+- to be defined
 description: ""</t>
         </is>
       </c>
@@ -6680,6 +6789,7 @@
       <c r="B136" t="inlineStr">
         <is>
           <t>- controversial
+  - to be discussed
 description: An, often numeric, theoretical (or otherwise abstract) representation of an Entity intended to generate Data describing one or more of its traits.</t>
         </is>
       </c>
@@ -6726,7 +6836,7 @@
       <c r="B137" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
@@ -6768,6 +6878,7 @@
       <c r="B138" t="inlineStr">
         <is>
           <t>- core
+- to be discussed
 description: Range of the Spectral Band.</t>
         </is>
       </c>
@@ -6810,7 +6921,7 @@
       <c r="B139" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
@@ -6886,6 +6997,7 @@
       <c r="B141" t="inlineStr">
         <is>
           <t>- high-impact
+- to be discussed
 description: Policy documents that represent the official written reference for a given Policy.</t>
         </is>
       </c>
@@ -6928,6 +7040,7 @@
       <c r="B142" t="inlineStr">
         <is>
           <t>- high-impact
+- to be discussed
 description: Deliberate system of guidelines to guide decisions and achieve rational outcomes, implemented as a procedure or protocol and typically promulgated through official written documents.</t>
         </is>
       </c>
@@ -6970,6 +7083,7 @@
       <c r="B143" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Spatial reference in the form of a label or code that identifies a Location.</t>
         </is>
       </c>
@@ -7016,6 +7130,7 @@
       <c r="B144" t="inlineStr">
         <is>
           <t>- high-impact
+- to be discussed
 description: Science domain dealing with technologies and methods of collecting and analyzing observations about the different Earth spheres.</t>
         </is>
       </c>
@@ -7063,6 +7178,7 @@
       <c r="B145" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Structured Data that is machine readable and can be automatically read and processed by a computer, such as HDF, NetCDF, CSV, JSON, XML, etc.</t>
         </is>
       </c>
@@ -7105,6 +7221,7 @@
       <c r="B146" t="inlineStr">
         <is>
           <t>- core
+- to be discussed
 description: Information used to determine geographic Location.</t>
         </is>
       </c>
@@ -7147,7 +7264,7 @@
       <c r="B147" t="inlineStr">
         <is>
           <t>- core
-- approved</t>
+- to be approved</t>
         </is>
       </c>
       <c r="C147" t="inlineStr"/>
@@ -7189,6 +7306,7 @@
       <c r="B148" t="inlineStr">
         <is>
           <t>- core
+  - to be defined
 description: ""</t>
         </is>
       </c>
@@ -7223,6 +7341,7 @@
       <c r="B149" t="inlineStr">
         <is>
           <t>- base
+  - to be approved
 description: Particular Place referenced by an identifier.</t>
         </is>
       </c>
@@ -7275,6 +7394,7 @@
       <c r="B150" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Device or instrument suited (through physical/chemical interaction) to measure one or more properties of a Phenomenon and thus collect factual/objective data.</t>
         </is>
       </c>
@@ -7323,6 +7443,7 @@
       <c r="B151" t="inlineStr">
         <is>
           <t>- core
+- to be approved
 description: Observation or model output representing regular intervals, specifying the length of the interval that determines the smallest event or process that can be resolved.</t>
         </is>
       </c>
@@ -7375,6 +7496,7 @@
       <c r="B152" t="inlineStr">
         <is>
           <t>- high-impact
+- to be discussed
 description: Well-established concept typically taught as the rational model of policy decision-making, representing an idealised view of the policy process.</t>
         </is>
       </c>

</xml_diff>